<commit_message>
data: publish 2026-10-28 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-28-182路.xlsx
+++ b/data/export/2026-10-28-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -743,32 +743,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +780,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +804,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +824,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -887,7 +895,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +934,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -937,7 +945,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -965,32 +973,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1010,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,17 +1034,17 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1042,13 +1054,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>83.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1125,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1164,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1159,7 +1175,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1236,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1286,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1347,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1397,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1458,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1508,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1516,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A35717D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1548,12 +1564,12 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1567,7 +1583,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1603,7 +1619,784 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-28 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-28-182路.xlsx
+++ b/data/export/2026-10-28-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC25"/>
+  <dimension ref="A1:AC31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>92.5</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:52</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1695,32 +1695,36 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>102分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1728,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1752,17 +1756,17 @@
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -1772,13 +1776,17 @@
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB11" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>102.0</t>
+        </is>
+      </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1847,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1878,7 +1886,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
@@ -1917,32 +1925,36 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>97分钟</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1950,7 +1962,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1974,37 +1986,37 @@
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>92.5</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2077,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2104,7 +2116,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
@@ -2176,7 +2188,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2215,7 +2227,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr">
@@ -2287,7 +2299,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2326,7 +2338,7 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr">
@@ -2402,7 +2414,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:52</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2517,7 +2529,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2628,7 +2640,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2667,7 +2679,7 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr">
@@ -2743,7 +2755,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2858,7 +2870,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2973,7 +2985,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3027,7 +3039,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3100,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3203,7 +3215,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3247,13 +3259,17 @@
       </c>
       <c r="AA24" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB24" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>102.0</t>
+        </is>
+      </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3330,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3368,6 +3384,684 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>92.5</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>2/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>3/14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>